<commit_message>
Prateleira: atualiza semana 14/09/2026 com Excel/PDF novos.
Inclui SOC CYRE3/BBDC4, Smart Hedge 3m, Call KO ampliadas, POP BITC11 e Compra de Put BOVA11; sem bid/delta no HTML.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/prateleira/operacoes/operacoes.xlsx
+++ b/prateleira/operacoes/operacoes.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PIMENTPA\Projects\Artes\clone-github\prateleira\operacoes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4FE46797-DBDB-4D0C-A947-08D1DE197848}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D98A4D1C-874F-4E17-BABD-CD23A85D6BEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15915" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{4BD3F994-188E-4AC8-9C05-940072856F1C}"/>
+    <workbookView xWindow="-15915" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{4BD3F994-188E-4AC8-9C05-940072856F1C}"/>
   </bookViews>
   <sheets>
     <sheet name="07.09.26" sheetId="1" r:id="rId1"/>
+    <sheet name="14.09.26" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="728" uniqueCount="205">
   <si>
     <t>SOC</t>
   </si>
@@ -519,6 +520,141 @@
   </si>
   <si>
     <t>38.03%</t>
+  </si>
+  <si>
+    <t>1.30%</t>
+  </si>
+  <si>
+    <t>-33.33%</t>
+  </si>
+  <si>
+    <t>1.80%</t>
+  </si>
+  <si>
+    <t>-37.40%</t>
+  </si>
+  <si>
+    <t>-38.00%</t>
+  </si>
+  <si>
+    <t>105.50%</t>
+  </si>
+  <si>
+    <t>88.00%</t>
+  </si>
+  <si>
+    <t>-44.00%</t>
+  </si>
+  <si>
+    <t>BBDC4</t>
+  </si>
+  <si>
+    <t>105.40%</t>
+  </si>
+  <si>
+    <t>-41.00%</t>
+  </si>
+  <si>
+    <t>4.40%</t>
+  </si>
+  <si>
+    <t>-79.46%</t>
+  </si>
+  <si>
+    <t>261.90%</t>
+  </si>
+  <si>
+    <t>-81.30%</t>
+  </si>
+  <si>
+    <t>SUZB3</t>
+  </si>
+  <si>
+    <t>126.17%</t>
+  </si>
+  <si>
+    <t>-63.00%</t>
+  </si>
+  <si>
+    <t>135.19%</t>
+  </si>
+  <si>
+    <t>-68.36%</t>
+  </si>
+  <si>
+    <t>126.43%</t>
+  </si>
+  <si>
+    <t>-59.33%</t>
+  </si>
+  <si>
+    <t>128.79%</t>
+  </si>
+  <si>
+    <t>-63.28%</t>
+  </si>
+  <si>
+    <t>SMAL11</t>
+  </si>
+  <si>
+    <t>116.00%</t>
+  </si>
+  <si>
+    <t>-33.00%</t>
+  </si>
+  <si>
+    <t>-3.60%</t>
+  </si>
+  <si>
+    <t>16.58%</t>
+  </si>
+  <si>
+    <t>129.28%</t>
+  </si>
+  <si>
+    <t>-4.00%</t>
+  </si>
+  <si>
+    <t>10.16%</t>
+  </si>
+  <si>
+    <t>123.19%</t>
+  </si>
+  <si>
+    <t>16.38%</t>
+  </si>
+  <si>
+    <t>119.90%</t>
+  </si>
+  <si>
+    <t>23.74%</t>
+  </si>
+  <si>
+    <t>POP</t>
+  </si>
+  <si>
+    <t>S CALL (0.5x)</t>
+  </si>
+  <si>
+    <t>BITC11</t>
+  </si>
+  <si>
+    <t>3.50%</t>
+  </si>
+  <si>
+    <t>-0.01%</t>
+  </si>
+  <si>
+    <t>COMPRA DE PUT</t>
+  </si>
+  <si>
+    <t>95.00%</t>
+  </si>
+  <si>
+    <t>-2.93%</t>
+  </si>
+  <si>
+    <t>-25.00%</t>
   </si>
 </sst>
 </file>
@@ -2198,4 +2334,1423 @@
     <oddFooter>&amp;L_x000D_&amp;1#&amp;"Aptos"&amp;10&amp;K000000 Internal Use Only</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2374A204-22BE-4DBC-BB7D-0412A8078370}">
+  <dimension ref="A1:J175"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="22.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.90625" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="7.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="3">
+        <v>46309</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="3">
+        <v>46296</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="3">
+        <v>46322</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="3">
+        <v>46323</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="3">
+        <v>46296</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" s="3">
+        <v>46308</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" s="3">
+        <v>46308</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" s="3">
+        <v>46304</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B14" s="4">
+        <v>46309</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B15" s="4">
+        <v>46322</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A29" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A30" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B30" s="3">
+        <v>46640</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A31" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B31" s="3">
+        <v>46640</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A32" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B32" s="3">
+        <v>46640</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A33" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B33" s="3">
+        <v>46643</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A34" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B34" s="3">
+        <v>47009</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A35" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B35" s="3">
+        <v>46644</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A36" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B36" s="3">
+        <v>47010</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A37" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B37" s="3">
+        <v>47010</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A38" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B38" s="3">
+        <v>47007</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A39" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="B39" s="4">
+        <v>46398</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A40" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B40" s="4">
+        <v>46398</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A41" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B41" s="4">
+        <v>46398</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A42" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B42" s="4">
+        <v>46398</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A58" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H58" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="I58" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A59" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B59" s="3">
+        <v>46791</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G59" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H59" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="I59" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A60" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B60" s="3">
+        <v>46398</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H60" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="I60" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A61" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="B61" s="4">
+        <v>46398</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H61" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="I61" s="2" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A75" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F75" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G75" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="H75" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I75" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J75" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A76" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B76" s="3">
+        <v>46643</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E76" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F76" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H76" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I76" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J76" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A77" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77" s="3">
+        <v>46458</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="E77" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F77" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="G77" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H77" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I77" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="J77" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A78" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B78" s="3">
+        <v>46643</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E78" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F78" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="G78" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H78" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I78" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J78" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A79" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B79" s="3">
+        <v>46643</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D79" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="E79" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F79" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="G79" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H79" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I79" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J79" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A80" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B80" s="3">
+        <v>46643</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D80" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E80" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F80" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="G80" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H80" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I80" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J80" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A81" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B81" s="3">
+        <v>46643</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="E81" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F81" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="G81" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H81" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I81" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J81" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A82" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B82" s="3">
+        <v>46643</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D82" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F82" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="G82" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H82" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I82" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J82" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A83" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B83" s="3">
+        <v>46643</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D83" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F83" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="G83" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H83" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I83" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J83" s="1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A84" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B84" s="3">
+        <v>46643</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="E84" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F84" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="G84" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H84" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I84" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J84" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A96" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E96" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="F96" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="G96" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A97" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B97" s="3">
+        <v>46339</v>
+      </c>
+      <c r="C97" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D97" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="E97" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F97" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="G97" s="1" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A98" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B98" s="4">
+        <v>46339</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="E98" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="F98" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="G98" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A99" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B99" s="4">
+        <v>46339</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D99" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="E99" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="F99" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="G99" s="2" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A100" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B100" s="4">
+        <v>46339</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D100" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="E100" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="F100" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="G100" s="2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A110" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A114" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B114" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C114" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D114" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E114" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="F114" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="G114" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A115" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B115" s="3">
+        <v>46366</v>
+      </c>
+      <c r="C115" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D115" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E115" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F115" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="G115" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A125" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="129" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A129" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B129" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C129" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D129" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E129" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F129" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G129" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H129" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="I129" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="130" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A130" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B130" s="3">
+        <v>46643</v>
+      </c>
+      <c r="C130" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D130" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E130" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="F130" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G130" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="H130" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="I130" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="138" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A138" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="142" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A142" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B142" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C142" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D142" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E142" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="F142" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="G142" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="143" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A143" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B143" s="3">
+        <v>46342</v>
+      </c>
+      <c r="C143" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D143" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="E143" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F143" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="G143" s="1" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="155" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A155" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="159" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A159" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B159" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C159" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="D159" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E159" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F159" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="160" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A160" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="B160" s="4">
+        <v>47016</v>
+      </c>
+      <c r="C160" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D160" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E160" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="F160" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A170" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A174" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B174" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C174" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D174" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="E174" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A175" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B175" s="4">
+        <v>46398</v>
+      </c>
+      <c r="C175" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="D175" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="E175" s="2" t="s">
+        <v>204</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Prateleira: atualiza precos de entrada das operacoes de premio.
Call KO 5%, Put KO 3,5%, One Touch BOVA11 1,2% conforme Excel.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/prateleira/operacoes/operacoes.xlsx
+++ b/prateleira/operacoes/operacoes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PIMENTPA\Projects\Artes\clone-github\prateleira\operacoes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D98A4D1C-874F-4E17-BABD-CD23A85D6BEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29C7E6C3-71E7-4EAF-8A3C-D64E7EA1FCFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15915" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{4BD3F994-188E-4AC8-9C05-940072856F1C}"/>
+    <workbookView xWindow="12975" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{4BD3F994-188E-4AC8-9C05-940072856F1C}"/>
   </bookViews>
   <sheets>
     <sheet name="07.09.26" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="728" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="203">
   <si>
     <t>SOC</t>
   </si>
@@ -603,16 +603,10 @@
     <t>-33.00%</t>
   </si>
   <si>
-    <t>-3.60%</t>
-  </si>
-  <si>
     <t>16.58%</t>
   </si>
   <si>
     <t>129.28%</t>
-  </si>
-  <si>
-    <t>-4.00%</t>
   </si>
   <si>
     <t>10.16%</t>
@@ -698,7 +692,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -710,6 +704,15 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3425,11 +3428,11 @@
       <c r="E97" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="F97" s="1" t="s">
+      <c r="F97" s="5">
+        <v>-0.05</v>
+      </c>
+      <c r="G97" s="1" t="s">
         <v>187</v>
-      </c>
-      <c r="G97" s="1" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.35">
@@ -3443,16 +3446,16 @@
         <v>64</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E98" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="F98" s="2" t="s">
-        <v>190</v>
+      <c r="F98" s="6">
+        <v>-0.05</v>
       </c>
       <c r="G98" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.35">
@@ -3466,16 +3469,16 @@
         <v>64</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E99" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="F99" s="2" t="s">
-        <v>190</v>
+      <c r="F99" s="6">
+        <v>-0.05</v>
       </c>
       <c r="G99" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.35">
@@ -3489,16 +3492,16 @@
         <v>64</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E100" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="F100" s="2" t="s">
-        <v>190</v>
+      <c r="F100" s="6">
+        <v>-0.05</v>
       </c>
       <c r="G100" s="2" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.35">
@@ -3545,8 +3548,8 @@
       <c r="E115" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="F115" s="1" t="s">
-        <v>139</v>
+      <c r="F115" s="7">
+        <v>-3.5000000000000003E-2</v>
       </c>
       <c r="G115" s="1" t="s">
         <v>140</v>
@@ -3659,8 +3662,8 @@
       <c r="E143" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F143" s="1" t="s">
-        <v>148</v>
+      <c r="F143" s="7">
+        <v>-1.2E-2</v>
       </c>
       <c r="G143" s="1" t="s">
         <v>149</v>
@@ -3668,7 +3671,7 @@
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="159" spans="1:6" ht="29" x14ac:dyDescent="0.35">
@@ -3679,7 +3682,7 @@
         <v>2</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D159" s="2" t="s">
         <v>46</v>
@@ -3693,7 +3696,7 @@
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A160" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B160" s="4">
         <v>47016</v>
@@ -3705,15 +3708,15 @@
         <v>64</v>
       </c>
       <c r="E160" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="F160" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.35">
@@ -3741,13 +3744,13 @@
         <v>46398</v>
       </c>
       <c r="C175" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="D175" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="E175" s="2" t="s">
         <v>202</v>
-      </c>
-      <c r="D175" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="E175" s="2" t="s">
-        <v>204</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Prateleira: atualiza semana 21/09 a partir do Excel.
</commit_message>
<xml_diff>
--- a/prateleira/operacoes/operacoes.xlsx
+++ b/prateleira/operacoes/operacoes.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PIMENTPA\Projects\Artes\clone-github\prateleira\operacoes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29C7E6C3-71E7-4EAF-8A3C-D64E7EA1FCFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56C7AA05-7956-43B2-8223-B200BC467FA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12975" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{4BD3F994-188E-4AC8-9C05-940072856F1C}"/>
+    <workbookView xWindow="-15915" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{4BD3F994-188E-4AC8-9C05-940072856F1C}"/>
   </bookViews>
   <sheets>
     <sheet name="07.09.26" sheetId="1" r:id="rId1"/>
     <sheet name="14.09.26" sheetId="2" r:id="rId2"/>
+    <sheet name="21.09.26" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1077" uniqueCount="232">
   <si>
     <t>SOC</t>
   </si>
@@ -649,6 +650,93 @@
   </si>
   <si>
     <t>-25.00%</t>
+  </si>
+  <si>
+    <t>1.20%</t>
+  </si>
+  <si>
+    <t>-33.32%</t>
+  </si>
+  <si>
+    <t>2.30%</t>
+  </si>
+  <si>
+    <t>-40.26%</t>
+  </si>
+  <si>
+    <t>-42.00%</t>
+  </si>
+  <si>
+    <t>VBBR3</t>
+  </si>
+  <si>
+    <t>-80.71%</t>
+  </si>
+  <si>
+    <t>137.50%</t>
+  </si>
+  <si>
+    <t>4.00%</t>
+  </si>
+  <si>
+    <t>-76.00%</t>
+  </si>
+  <si>
+    <t>SBSP3</t>
+  </si>
+  <si>
+    <t>136.88%</t>
+  </si>
+  <si>
+    <t>-57.00%</t>
+  </si>
+  <si>
+    <t>COMPRA DE CALL SPREAD</t>
+  </si>
+  <si>
+    <t>B CALL</t>
+  </si>
+  <si>
+    <t>105.00%</t>
+  </si>
+  <si>
+    <t>-2.00%</t>
+  </si>
+  <si>
+    <t>26.02%</t>
+  </si>
+  <si>
+    <t>COLLAR</t>
+  </si>
+  <si>
+    <t>MELI34</t>
+  </si>
+  <si>
+    <t>127.00%</t>
+  </si>
+  <si>
+    <t>3.00%</t>
+  </si>
+  <si>
+    <t>-70.00%</t>
+  </si>
+  <si>
+    <t>LREN3</t>
+  </si>
+  <si>
+    <t>125.00%</t>
+  </si>
+  <si>
+    <t>123.00%</t>
+  </si>
+  <si>
+    <t>-73.00%</t>
+  </si>
+  <si>
+    <t>-55.50%</t>
+  </si>
+  <si>
+    <t>128.00%</t>
   </si>
 </sst>
 </file>
@@ -3756,4 +3844,1328 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BC8F196-C523-4A89-A0DA-31289464916B}">
+  <dimension ref="A1:J159"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="10.26953125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="3">
+        <v>46330</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="3">
+        <v>46303</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="3">
+        <v>46315</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" s="3">
+        <v>46315</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="3">
+        <v>46314</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B11" s="3">
+        <v>46316</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="B12" s="3">
+        <v>46331</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A26" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B27" s="3">
+        <v>46647</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B28" s="3">
+        <v>46647</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A29" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B29" s="3">
+        <v>46647</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A30" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3">
+        <v>46650</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A31" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B31" s="3">
+        <v>47016</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A32" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B32" s="3">
+        <v>46651</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A33" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B33" s="3">
+        <v>47017</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A34" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B34" s="3">
+        <v>47017</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A35" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B35" s="3">
+        <v>47014</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A36" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36" s="3">
+        <v>46405</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A37" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B37" s="3">
+        <v>46405</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A38" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B38" s="3">
+        <v>46405</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A39" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B39" s="4">
+        <v>46465</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A40" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B40" s="4">
+        <v>46650</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A54" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H54" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="I54" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A55" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B55" s="3">
+        <v>46798</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H55" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="I55" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A56" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B56" s="3">
+        <v>46405</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H56" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="I56" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A68" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E68" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F68" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="H68" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I68" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J68" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A69" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B69" s="3">
+        <v>46650</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E69" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F69" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="G69" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H69" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I69" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J69" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A70" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B70" s="3">
+        <v>46465</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F70" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="G70" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H70" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I70" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="J70" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A71" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B71" s="3">
+        <v>46650</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="G71" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H71" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I71" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J71" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A72" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B72" s="3">
+        <v>46650</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="E72" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H72" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I72" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J72" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A73" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B73" s="3">
+        <v>46650</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E73" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="G73" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H73" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I73" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J73" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A74" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B74" s="3">
+        <v>46650</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="E74" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F74" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="G74" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H74" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I74" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J74" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A75" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B75" s="3">
+        <v>46650</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D75" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="E75" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F75" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="G75" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H75" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I75" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J75" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A76" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B76" s="3">
+        <v>46650</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E76" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F76" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H76" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I76" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J76" s="1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A77" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B77" s="3">
+        <v>46650</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="E77" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F77" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="G77" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H77" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I77" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J77" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A78" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="B78" s="4">
+        <v>46650</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F78" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="G78" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="H78" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="I78" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="J78" s="2" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A92" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E92" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="F92" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="G92" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A93" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B93" s="3">
+        <v>46373</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D93" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E93" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F93" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="G93" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A105" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="109" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A109" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B109" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C109" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D109" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E109" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F109" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G109" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H109" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="I109" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="110" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A110" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B110" s="3">
+        <v>46650</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D110" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E110" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="F110" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G110" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="H110" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="I110" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A120" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A124" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B124" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C124" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D124" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="E124" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A125" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B125" s="3">
+        <v>46405</v>
+      </c>
+      <c r="C125" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="D125" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="E125" s="1" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A135" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A139" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B139" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C139" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="D139" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E139" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="F139" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A140" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B140" s="3">
+        <v>46323</v>
+      </c>
+      <c r="C140" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D140" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="E140" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="F140" s="1" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A150" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A154" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B154" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C154" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D154" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E154" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F154" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="155" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A155" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="B155" s="4">
+        <v>46650</v>
+      </c>
+      <c r="C155" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D155" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="E155" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="F155" s="2" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="156" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A156" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B156" s="4">
+        <v>46650</v>
+      </c>
+      <c r="C156" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D156" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="E156" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="F156" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="157" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A157" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B157" s="4">
+        <v>46650</v>
+      </c>
+      <c r="C157" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D157" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="E157" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="F157" s="2" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="158" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A158" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B158" s="4">
+        <v>46464</v>
+      </c>
+      <c r="C158" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D158" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E158" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="F158" s="2" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="159" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A159" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B159" s="4">
+        <v>46647</v>
+      </c>
+      <c r="C159" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D159" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="E159" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="F159" s="2" t="s">
+        <v>177</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Prateleira: atualiza semana 28/09 a partir do Excel e PDF.
</commit_message>
<xml_diff>
--- a/prateleira/operacoes/operacoes.xlsx
+++ b/prateleira/operacoes/operacoes.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PIMENTPA\Projects\Artes\clone-github\prateleira\operacoes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F29A7D5F-1569-418E-8DA1-F19E34B039BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0185729-7B97-43A8-9C93-2B5D6431C5AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12975" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{4BD3F994-188E-4AC8-9C05-940072856F1C}"/>
+    <workbookView xWindow="-15915" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{4BD3F994-188E-4AC8-9C05-940072856F1C}"/>
   </bookViews>
   <sheets>
     <sheet name="07.09.26" sheetId="1" r:id="rId1"/>
     <sheet name="14.09.26" sheetId="2" r:id="rId2"/>
     <sheet name="21.09.26" sheetId="3" r:id="rId3"/>
+    <sheet name="28.09.26" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1074" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1426" uniqueCount="260">
   <si>
     <t>SOC</t>
   </si>
@@ -734,6 +735,93 @@
   </si>
   <si>
     <t>128.00%</t>
+  </si>
+  <si>
+    <t>1.10%</t>
+  </si>
+  <si>
+    <t>-32.59%</t>
+  </si>
+  <si>
+    <t>1.91%</t>
+  </si>
+  <si>
+    <t>1.17%</t>
+  </si>
+  <si>
+    <t>M1TA34</t>
+  </si>
+  <si>
+    <t>107.45%</t>
+  </si>
+  <si>
+    <t>4.70%</t>
+  </si>
+  <si>
+    <t>-68.73%</t>
+  </si>
+  <si>
+    <t>3.60%</t>
+  </si>
+  <si>
+    <t>-71.07%</t>
+  </si>
+  <si>
+    <t>3.08%</t>
+  </si>
+  <si>
+    <t>-83.00%</t>
+  </si>
+  <si>
+    <t>-56.66%</t>
+  </si>
+  <si>
+    <t>-80.00%</t>
+  </si>
+  <si>
+    <t>6.14%</t>
+  </si>
+  <si>
+    <t>-75.00%</t>
+  </si>
+  <si>
+    <t>SMAB11</t>
+  </si>
+  <si>
+    <t>163.55%</t>
+  </si>
+  <si>
+    <t>-88.75%</t>
+  </si>
+  <si>
+    <t>-29.00%</t>
+  </si>
+  <si>
+    <t>P2LT34</t>
+  </si>
+  <si>
+    <t>180.00%</t>
+  </si>
+  <si>
+    <t>-51.00%</t>
+  </si>
+  <si>
+    <t>-2.00%</t>
+  </si>
+  <si>
+    <t>112.00%</t>
+  </si>
+  <si>
+    <t>-54.93%</t>
+  </si>
+  <si>
+    <t>124.00%</t>
+  </si>
+  <si>
+    <t>-68.00%</t>
+  </si>
+  <si>
+    <t>-65.12%</t>
   </si>
 </sst>
 </file>
@@ -5165,4 +5253,1326 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D728F6DC-D0DF-483D-B9A9-BCB1E9A6DB89}">
+  <dimension ref="A1:J136"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="22.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.90625" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="7.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="3">
+        <v>46337</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" s="3">
+        <v>46322</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="3">
+        <v>46322</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B9" s="3">
+        <v>46323</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="B10" s="3">
+        <v>46338</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="B11" s="4">
+        <v>46335</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B26" s="3">
+        <v>46654</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B27" s="3">
+        <v>46654</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B28" s="3">
+        <v>46654</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A29" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B29" s="3">
+        <v>46657</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A30" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3">
+        <v>47023</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A31" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B31" s="3">
+        <v>46658</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A32" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B32" s="3">
+        <v>47024</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A33" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B33" s="3">
+        <v>47024</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A34" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B34" s="3">
+        <v>47021</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A35" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B35" s="3">
+        <v>46412</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A36" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B36" s="3">
+        <v>46412</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A37" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B37" s="3">
+        <v>46412</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A38" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B38" s="3">
+        <v>46475</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A39" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B39" s="3">
+        <v>46657</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="G39" s="1" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A40" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="B40" s="3">
+        <v>46657</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A41" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B41" s="4">
+        <v>46654</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A55" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="I55" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A56" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B56" s="3">
+        <v>46805</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H56" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="I56" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A57" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B57" s="3">
+        <v>46412</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G57" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H57" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="I57" s="1" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A69" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E69" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F69" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G69" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="H69" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I69" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J69" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A70" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B70" s="3">
+        <v>46657</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F70" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="G70" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H70" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I70" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J70" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A71" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B71" s="3">
+        <v>46475</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="G71" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H71" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I71" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="J71" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A72" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B72" s="3">
+        <v>46657</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E72" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H72" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I72" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J72" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A73" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B73" s="3">
+        <v>46657</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="E73" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="G73" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H73" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I73" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J73" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A74" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B74" s="3">
+        <v>46657</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E74" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F74" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="G74" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H74" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I74" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J74" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A75" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B75" s="3">
+        <v>46657</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D75" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="E75" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F75" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="G75" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H75" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I75" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J75" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A76" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B76" s="3">
+        <v>46657</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="E76" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F76" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H76" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I76" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J76" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A77" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B77" s="3">
+        <v>46657</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E77" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F77" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="G77" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H77" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I77" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J77" s="1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A78" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B78" s="3">
+        <v>46657</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="E78" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F78" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="G78" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H78" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I78" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J78" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A79" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="B79" s="4">
+        <v>46654</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="E79" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F79" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="G79" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="H79" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="I79" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="J79" s="2" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A91" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E91" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F91" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G91" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H91" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="I91" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A92" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B92" s="3">
+        <v>46657</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D92" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E92" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="F92" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G92" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="H92" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="I92" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A104" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="E104" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A105" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B105" s="3">
+        <v>46412</v>
+      </c>
+      <c r="C105" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="D105" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="E105" s="1" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A113" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A117" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B117" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C117" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="D117" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E117" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="F117" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A118" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118" s="3">
+        <v>46331</v>
+      </c>
+      <c r="C118" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D118" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="E118" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="F118" s="1" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A126" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A130" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B130" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C130" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D130" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E130" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F130" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A131" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="B131" s="3">
+        <v>46657</v>
+      </c>
+      <c r="C131" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D131" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="E131" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="F131" s="1" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A132" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="B132" s="3">
+        <v>46657</v>
+      </c>
+      <c r="C132" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D132" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="E132" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="F132" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A133" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B133" s="3">
+        <v>46657</v>
+      </c>
+      <c r="C133" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D133" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="E133" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="F133" s="1" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A134" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B134" s="3">
+        <v>46471</v>
+      </c>
+      <c r="C134" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D134" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="E134" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F134" s="1" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A135" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B135" s="3">
+        <v>46654</v>
+      </c>
+      <c r="C135" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D135" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="E135" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="F135" s="1" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A136" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B136" s="4">
+        <v>46469</v>
+      </c>
+      <c r="C136" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D136" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="E136" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="F136" s="2" t="s">
+        <v>259</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Prateleira: atualiza semana 19/10 a partir do Excel.
</commit_message>
<xml_diff>
--- a/prateleira/operacoes/operacoes.xlsx
+++ b/prateleira/operacoes/operacoes.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PIMENTPA\Projects\Artes\clone-github\prateleira\operacoes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0185729-7B97-43A8-9C93-2B5D6431C5AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2ED002E-2DDF-4353-AA1E-EF9C6B4861DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15915" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{4BD3F994-188E-4AC8-9C05-940072856F1C}"/>
+    <workbookView xWindow="-15915" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{4BD3F994-188E-4AC8-9C05-940072856F1C}"/>
   </bookViews>
   <sheets>
     <sheet name="07.09.26" sheetId="1" r:id="rId1"/>
     <sheet name="14.09.26" sheetId="2" r:id="rId2"/>
     <sheet name="21.09.26" sheetId="3" r:id="rId3"/>
     <sheet name="28.09.26" sheetId="4" r:id="rId4"/>
+    <sheet name="19.10.26" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1426" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1692" uniqueCount="312">
   <si>
     <t>SOC</t>
   </si>
@@ -822,6 +823,162 @@
   </si>
   <si>
     <t>-65.12%</t>
+  </si>
+  <si>
+    <t>-49.40%</t>
+  </si>
+  <si>
+    <t>3.90%</t>
+  </si>
+  <si>
+    <t>-54.00%</t>
+  </si>
+  <si>
+    <t>103.56%</t>
+  </si>
+  <si>
+    <t>1.05%</t>
+  </si>
+  <si>
+    <t>110.06%</t>
+  </si>
+  <si>
+    <t>-26.80%</t>
+  </si>
+  <si>
+    <t>106.29%</t>
+  </si>
+  <si>
+    <t>-35.21%</t>
+  </si>
+  <si>
+    <t>BRAV3</t>
+  </si>
+  <si>
+    <t>106.18%</t>
+  </si>
+  <si>
+    <t>-34.15%</t>
+  </si>
+  <si>
+    <t>104.50%</t>
+  </si>
+  <si>
+    <t>-43.44%</t>
+  </si>
+  <si>
+    <t>GGBR4</t>
+  </si>
+  <si>
+    <t>-41.16%</t>
+  </si>
+  <si>
+    <t>AMZO34</t>
+  </si>
+  <si>
+    <t>-41.91%</t>
+  </si>
+  <si>
+    <t>-41.24%</t>
+  </si>
+  <si>
+    <t>-74.56%</t>
+  </si>
+  <si>
+    <t>-76.76%</t>
+  </si>
+  <si>
+    <t>132.00%</t>
+  </si>
+  <si>
+    <t>-73.40%</t>
+  </si>
+  <si>
+    <t>126.00%</t>
+  </si>
+  <si>
+    <t>-71.02%</t>
+  </si>
+  <si>
+    <t>-73.83%</t>
+  </si>
+  <si>
+    <t>-85.14%</t>
+  </si>
+  <si>
+    <t>28.76%</t>
+  </si>
+  <si>
+    <t>25.50%</t>
+  </si>
+  <si>
+    <t>41.40%</t>
+  </si>
+  <si>
+    <t>-60.00%</t>
+  </si>
+  <si>
+    <t>116.83%</t>
+  </si>
+  <si>
+    <t>-55.28%</t>
+  </si>
+  <si>
+    <t>-61.00%</t>
+  </si>
+  <si>
+    <t>119.35%</t>
+  </si>
+  <si>
+    <t>3.14%</t>
+  </si>
+  <si>
+    <t>-58.60%</t>
+  </si>
+  <si>
+    <t>MGLU3</t>
+  </si>
+  <si>
+    <t>-77.00%</t>
+  </si>
+  <si>
+    <t>111.00%</t>
+  </si>
+  <si>
+    <t>-64.65%</t>
+  </si>
+  <si>
+    <t>EQTL3</t>
+  </si>
+  <si>
+    <t>108.00%</t>
+  </si>
+  <si>
+    <t>ASAI3</t>
+  </si>
+  <si>
+    <t>102.00%</t>
+  </si>
+  <si>
+    <t>118.00%</t>
+  </si>
+  <si>
+    <t>13.00%</t>
+  </si>
+  <si>
+    <t>MOVI3</t>
+  </si>
+  <si>
+    <t>9.00%</t>
+  </si>
+  <si>
+    <t>117.00%</t>
+  </si>
+  <si>
+    <t>14.00%</t>
+  </si>
+  <si>
+    <t>-63.67%</t>
   </si>
 </sst>
 </file>
@@ -865,7 +1022,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -887,6 +1044,9 @@
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6575,4 +6735,1032 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA2DB65C-88C9-41DB-823D-72C5178556C6}">
+  <dimension ref="A1:J133"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="10.26953125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="3">
+        <v>46343</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="3">
+        <v>46343</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B8" s="3">
+        <v>46342</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="3">
+        <v>46339</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="3">
+        <v>46339</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="B11" s="3">
+        <v>46356</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="4">
+        <v>46356</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="B13" s="4">
+        <v>46342</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="B14" s="4">
+        <v>46342</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B15" s="4">
+        <v>46342</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A31" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A32" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B32" s="3">
+        <v>46675</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A33" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B33" s="3">
+        <v>46675</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A34" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B34" s="3">
+        <v>46675</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A35" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B35" s="3">
+        <v>46490</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A36" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36" s="3">
+        <v>46490</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A37" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B37" s="3">
+        <v>46490</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A38" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B38" s="3">
+        <v>46490</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A39" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B39" s="3">
+        <v>46490</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="G39" s="1" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A53" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="H53" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I53" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J53" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A54" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B54" s="3">
+        <v>46678</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H54" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I54" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="J54" s="1" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A55" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B55" s="3">
+        <v>46678</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H55" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I55" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J55" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A56" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B56" s="3">
+        <v>46678</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H56" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I56" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J56" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A70" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A71" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B71" s="3">
+        <v>46352</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="E71" s="7">
+        <v>-3.1E-2</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A72" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="B72" s="3">
+        <v>46370</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="E72" s="7">
+        <v>-4.8399999999999999E-2</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A73" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B73" s="4">
+        <v>46370</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="E73" s="8">
+        <v>-4.5999999999999999E-2</v>
+      </c>
+      <c r="F73" s="2" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A89" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E89" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F89" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A90" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B90" s="3">
+        <v>46492</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D90" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="E90" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F90" s="1" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A91" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B91" s="3">
+        <v>46675</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D91" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="E91" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F91" s="1" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A92" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B92" s="3">
+        <v>46492</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D92" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="E92" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F92" s="1" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A93" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B93" s="3">
+        <v>46675</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D93" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="E93" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="F93" s="1" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A94" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B94" s="3">
+        <v>46675</v>
+      </c>
+      <c r="C94" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D94" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="E94" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="F94" s="1" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A95" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="B95" s="3">
+        <v>46400</v>
+      </c>
+      <c r="C95" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D95" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E95" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F95" s="1" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A96" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B96" s="3">
+        <v>46400</v>
+      </c>
+      <c r="C96" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D96" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="E96" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F96" s="1" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A97" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="B97" s="3">
+        <v>46400</v>
+      </c>
+      <c r="C97" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D97" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="E97" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F97" s="1" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A109" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A113" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B113" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C113" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D113" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E113" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="F113" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="G113" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A114" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="B114" s="3">
+        <v>46371</v>
+      </c>
+      <c r="C114" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="D114" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="E114" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F114" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="G114" s="1" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A115" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="B115" s="3">
+        <v>46371</v>
+      </c>
+      <c r="C115" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="D115" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="E115" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F115" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="G115" s="1" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A116" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B116" s="3">
+        <v>46371</v>
+      </c>
+      <c r="C116" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="D116" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="E116" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F116" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="G116" s="1" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="128" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A128" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A132" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B132" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C132" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="D132" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E132" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F132" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A133" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="B133" s="3">
+        <v>46675</v>
+      </c>
+      <c r="C133" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D133" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E133" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="F133" s="1" t="s">
+        <v>311</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Prateleira: atualiza parametros da aba 19.10 a partir do Excel.
</commit_message>
<xml_diff>
--- a/prateleira/operacoes/operacoes.xlsx
+++ b/prateleira/operacoes/operacoes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PIMENTPA\Projects\Artes\clone-github\prateleira\operacoes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2ED002E-2DDF-4353-AA1E-EF9C6B4861DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53304EEA-B49F-41CC-9B9C-15B30E01E882}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-15915" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{4BD3F994-188E-4AC8-9C05-940072856F1C}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1692" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1671" uniqueCount="311">
   <si>
     <t>SOC</t>
   </si>
@@ -825,42 +825,15 @@
     <t>-65.12%</t>
   </si>
   <si>
-    <t>-49.40%</t>
-  </si>
-  <si>
-    <t>3.90%</t>
-  </si>
-  <si>
-    <t>-54.00%</t>
-  </si>
-  <si>
     <t>103.56%</t>
   </si>
   <si>
     <t>1.05%</t>
   </si>
   <si>
-    <t>110.06%</t>
-  </si>
-  <si>
-    <t>-26.80%</t>
-  </si>
-  <si>
-    <t>106.29%</t>
-  </si>
-  <si>
-    <t>-35.21%</t>
-  </si>
-  <si>
     <t>BRAV3</t>
   </si>
   <si>
-    <t>106.18%</t>
-  </si>
-  <si>
-    <t>-34.15%</t>
-  </si>
-  <si>
     <t>104.50%</t>
   </si>
   <si>
@@ -882,9 +855,6 @@
     <t>-41.24%</t>
   </si>
   <si>
-    <t>-74.56%</t>
-  </si>
-  <si>
     <t>-76.76%</t>
   </si>
   <si>
@@ -909,12 +879,6 @@
     <t>28.76%</t>
   </si>
   <si>
-    <t>25.50%</t>
-  </si>
-  <si>
-    <t>41.40%</t>
-  </si>
-  <si>
     <t>-60.00%</t>
   </si>
   <si>
@@ -978,7 +942,40 @@
     <t>14.00%</t>
   </si>
   <si>
-    <t>-63.67%</t>
+    <t>112.49%</t>
+  </si>
+  <si>
+    <t>-26.62%</t>
+  </si>
+  <si>
+    <t>114.56%</t>
+  </si>
+  <si>
+    <t>-26.67%</t>
+  </si>
+  <si>
+    <t>113.29%</t>
+  </si>
+  <si>
+    <t>-27.82%</t>
+  </si>
+  <si>
+    <t>106.85%</t>
+  </si>
+  <si>
+    <t>-33.67%</t>
+  </si>
+  <si>
+    <t>Triplo Retorno KO</t>
+  </si>
+  <si>
+    <t>COMPRA DE CS</t>
+  </si>
+  <si>
+    <t>17.40%</t>
+  </si>
+  <si>
+    <t>35.63%</t>
   </si>
 </sst>
 </file>
@@ -6739,1026 +6736,1323 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA2DB65C-88C9-41DB-823D-72C5178556C6}">
-  <dimension ref="A1:J133"/>
+  <dimension ref="A1:K84"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B6" s="3">
-        <v>46343</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>35</v>
+      <c r="C2" s="3">
+        <v>46345</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="3">
+        <v>46345</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C4" s="3">
+        <v>46344</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="3">
+        <v>46345</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="C6" s="3">
+        <v>46359</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>35</v>
+        <v>305</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>10</v>
+        <v>305</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>239</v>
+        <v>10</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A7" s="1"/>
+      <c r="B7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="4">
+        <v>46358</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A8" s="1"/>
+      <c r="B8" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="C8" s="4">
+        <v>46344</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A9" s="1"/>
+      <c r="B9" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C9" s="4">
+        <v>46344</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A10" s="1"/>
+      <c r="B10" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C10" s="4">
+        <v>46344</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+    </row>
+    <row r="12" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="3">
+        <v>46679</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A14" s="1"/>
+      <c r="B14" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C14" s="3">
+        <v>46679</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C15" s="3">
+        <v>46679</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
+      <c r="K15" s="1"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A16" s="1"/>
+      <c r="B16" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="3">
+        <v>46492</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A17" s="1"/>
+      <c r="B17" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C17" s="3">
+        <v>46492</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C18" s="3">
+        <v>46492</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A19" s="1"/>
+      <c r="B19" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="3">
-        <v>46343</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>261</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="B8" s="3">
-        <v>46342</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>263</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>263</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" s="3">
-        <v>46339</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B10" s="3">
-        <v>46339</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>267</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>267</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
-        <v>269</v>
-      </c>
-      <c r="B11" s="3">
+      <c r="C19" s="3">
+        <v>46492</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+      <c r="K19" s="1"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A20" s="1"/>
+      <c r="B20" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C20" s="3">
+        <v>46492</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
+      <c r="K20" s="1"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+      <c r="J21" s="1"/>
+      <c r="K21" s="1"/>
+    </row>
+    <row r="22" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A22" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A23" s="1"/>
+      <c r="B23" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" s="3">
+        <v>46680</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="J23" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="K23" s="1" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A24" s="1"/>
+      <c r="B24" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C24" s="3">
+        <v>46680</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="K24" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A25" s="1"/>
+      <c r="B25" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C25" s="3">
+        <v>46680</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="K25" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A26" s="1"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1"/>
+      <c r="K26" s="1"/>
+    </row>
+    <row r="27" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+      <c r="A27" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H27" s="1"/>
+      <c r="I27" s="1"/>
+      <c r="J27" s="1"/>
+      <c r="K27" s="1"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A28" s="1"/>
+      <c r="B28" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="C28" s="3">
         <v>46356</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>270</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>270</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B12" s="4">
-        <v>46356</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="B13" s="4">
-        <v>46342</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="B14" s="4">
-        <v>46342</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G14" s="2" t="s">
+      <c r="D28" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="F28" s="7">
+        <v>-4.8000000000000001E-2</v>
+      </c>
+      <c r="G28" s="1" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A15" s="2" t="s">
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+      <c r="J28" s="1"/>
+      <c r="K28" s="1"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A29" s="1"/>
+      <c r="B29" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="C29" s="3">
+        <v>46372</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="F29" s="7">
+        <v>-4.8000000000000001E-2</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="H29" s="1"/>
+      <c r="I29" s="1"/>
+      <c r="J29" s="1"/>
+      <c r="K29" s="1"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A30" s="1"/>
+      <c r="B30" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C30" s="4">
+        <v>46372</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="F30" s="8">
+        <v>-4.2000000000000003E-2</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
+      <c r="J30" s="1"/>
+      <c r="K30" s="1"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A31" s="1"/>
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+      <c r="I31" s="1"/>
+      <c r="J31" s="1"/>
+      <c r="K31" s="1"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A32" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H32" s="1"/>
+      <c r="I32" s="1"/>
+      <c r="J32" s="1"/>
+      <c r="K32" s="1"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A33" s="1"/>
+      <c r="B33" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B15" s="4">
-        <v>46342</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G15" s="2" t="s">
+      <c r="C33" s="3">
+        <v>46496</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="H33" s="1"/>
+      <c r="I33" s="1"/>
+      <c r="J33" s="1"/>
+      <c r="K33" s="1"/>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A34" s="1"/>
+      <c r="B34" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C34" s="3">
+        <v>46679</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="G34" s="1" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A31" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A32" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B32" s="3">
-        <v>46675</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="G32" s="1" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A33" s="1" t="s">
+      <c r="H34" s="1"/>
+      <c r="I34" s="1"/>
+      <c r="J34" s="1"/>
+      <c r="K34" s="1"/>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A35" s="1"/>
+      <c r="B35" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B33" s="3">
-        <v>46675</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="G33" s="1" t="s">
+      <c r="C35" s="3">
+        <v>46496</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E35" s="1" t="s">
         <v>279</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A34" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="B34" s="3">
-        <v>46675</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="G34" s="1" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A35" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B35" s="3">
-        <v>46490</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>117</v>
-      </c>
       <c r="F35" s="1" t="s">
-        <v>223</v>
+        <v>27</v>
       </c>
       <c r="G35" s="1" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A36" s="1" t="s">
+      <c r="H35" s="1"/>
+      <c r="I35" s="1"/>
+      <c r="J35" s="1"/>
+      <c r="K35" s="1"/>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A36" s="1"/>
+      <c r="B36" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B36" s="3">
-        <v>46490</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>10</v>
+      <c r="C36" s="3">
+        <v>46679</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E36" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="G36" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="F36" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="G36" s="1" t="s">
+      <c r="H36" s="1"/>
+      <c r="I36" s="1"/>
+      <c r="J36" s="1"/>
+      <c r="K36" s="1"/>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A37" s="1"/>
+      <c r="B37" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C37" s="3">
+        <v>46679</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E37" s="1" t="s">
         <v>282</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A37" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B37" s="3">
-        <v>46490</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E37" s="1" t="s">
+      <c r="F37" s="1" t="s">
         <v>283</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>223</v>
       </c>
       <c r="G37" s="1" t="s">
         <v>284</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A38" s="1" t="s">
+      <c r="H37" s="1"/>
+      <c r="I37" s="1"/>
+      <c r="J37" s="1"/>
+      <c r="K37" s="1"/>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A38" s="1"/>
+      <c r="B38" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="C38" s="3">
+        <v>46402</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="H38" s="1"/>
+      <c r="I38" s="1"/>
+      <c r="J38" s="1"/>
+      <c r="K38" s="1"/>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A39" s="1"/>
+      <c r="B39" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B38" s="3">
-        <v>46490</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E38" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="G38" s="1" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A39" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="B39" s="3">
-        <v>46490</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>10</v>
+      <c r="C39" s="3">
+        <v>46402</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>143</v>
+        <v>287</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>223</v>
+        <v>98</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A53" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="H39" s="1"/>
+      <c r="I39" s="1"/>
+      <c r="J39" s="1"/>
+      <c r="K39" s="1"/>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A40" s="1"/>
+      <c r="B40" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="C40" s="3">
+        <v>46402</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="H40" s="1"/>
+      <c r="I40" s="1"/>
+      <c r="J40" s="1"/>
+      <c r="K40" s="1"/>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A41" s="1"/>
+      <c r="B41" s="1"/>
+      <c r="C41" s="1"/>
+      <c r="D41" s="1"/>
+      <c r="E41" s="1"/>
+      <c r="F41" s="1"/>
+      <c r="G41" s="1"/>
+      <c r="H41" s="1"/>
+      <c r="I41" s="1"/>
+      <c r="J41" s="1"/>
+      <c r="K41" s="1"/>
+    </row>
+    <row r="42" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A42" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B42" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B53" s="2" t="s">
+      <c r="C42" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C53" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="D53" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E53" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="F53" s="2" t="s">
+      <c r="D42" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E42" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G53" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="H53" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="I53" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="J53" s="2" t="s">
+      <c r="F42" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="H42" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A54" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B54" s="3">
-        <v>46678</v>
-      </c>
-      <c r="C54" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="D54" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="E54" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="G54" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="H54" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="I54" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="J54" s="1" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A55" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="B55" s="3">
-        <v>46678</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="E55" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="F55" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="G55" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="H55" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="I55" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="J55" s="1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A56" s="1" t="s">
+      <c r="I42" s="1"/>
+      <c r="J42" s="1"/>
+      <c r="K42" s="1"/>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A43" s="1"/>
+      <c r="B43" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="C43" s="3">
+        <v>46373</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="G43" s="7">
+        <v>-4.4999999999999998E-2</v>
+      </c>
+      <c r="H43" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="I43" s="1"/>
+      <c r="J43" s="1"/>
+      <c r="K43" s="1"/>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A44" s="1"/>
+      <c r="B44" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="C44" s="3">
+        <v>46373</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="G44" s="7">
+        <v>-4.4999999999999998E-2</v>
+      </c>
+      <c r="H44" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="I44" s="1"/>
+      <c r="J44" s="1"/>
+      <c r="K44" s="1"/>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A45" s="1"/>
+      <c r="B45" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="B56" s="3">
-        <v>46678</v>
-      </c>
-      <c r="C56" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="D56" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="E56" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="F56" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="G56" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="H56" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="I56" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="J56" s="1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A66" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A70" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B70" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C70" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="D70" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E70" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="F70" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A71" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="B71" s="3">
-        <v>46352</v>
-      </c>
-      <c r="C71" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="D71" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E71" s="7">
-        <v>-3.1E-2</v>
-      </c>
-      <c r="F71" s="1" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A72" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="B72" s="3">
-        <v>46370</v>
-      </c>
-      <c r="C72" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="D72" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E72" s="7">
-        <v>-4.8399999999999999E-2</v>
-      </c>
-      <c r="F72" s="1" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A73" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="B73" s="4">
-        <v>46370</v>
-      </c>
-      <c r="C73" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="E73" s="8">
-        <v>-4.5999999999999999E-2</v>
-      </c>
-      <c r="F73" s="2" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A85" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A89" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B89" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C89" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D89" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E89" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F89" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A90" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B90" s="3">
-        <v>46492</v>
-      </c>
-      <c r="C90" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D90" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="E90" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="F90" s="1" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A91" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B91" s="3">
-        <v>46675</v>
-      </c>
-      <c r="C91" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D91" s="1" t="s">
-        <v>257</v>
-      </c>
-      <c r="E91" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="F91" s="1" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A92" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="B92" s="3">
-        <v>46492</v>
-      </c>
-      <c r="C92" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D92" s="1" t="s">
-        <v>291</v>
-      </c>
-      <c r="E92" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="F92" s="1" t="s">
+      <c r="C45" s="3">
+        <v>46373</v>
+      </c>
+      <c r="D45" s="1" t="s">
         <v>292</v>
       </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A93" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="B93" s="3">
-        <v>46675</v>
-      </c>
-      <c r="C93" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D93" s="1" t="s">
-        <v>257</v>
-      </c>
-      <c r="E93" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="F93" s="1" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A94" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B94" s="3">
-        <v>46675</v>
-      </c>
-      <c r="C94" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D94" s="1" t="s">
-        <v>294</v>
-      </c>
-      <c r="E94" s="1" t="s">
-        <v>295</v>
-      </c>
-      <c r="F94" s="1" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A95" s="1" t="s">
+      <c r="E45" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="B95" s="3">
-        <v>46400</v>
-      </c>
-      <c r="C95" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D95" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="E95" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="F95" s="1" t="s">
+      <c r="F45" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="G45" s="7">
+        <v>-4.4999999999999998E-2</v>
+      </c>
+      <c r="H45" s="1" t="s">
         <v>298</v>
       </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A96" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B96" s="3">
-        <v>46400</v>
-      </c>
-      <c r="C96" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D96" s="1" t="s">
-        <v>299</v>
-      </c>
-      <c r="E96" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="F96" s="1" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A97" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="B97" s="3">
-        <v>46400</v>
-      </c>
-      <c r="C97" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D97" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="E97" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="F97" s="1" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A109" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="113" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A113" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B113" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C113" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="D113" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E113" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="F113" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="G113" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A114" s="1" t="s">
-        <v>303</v>
-      </c>
-      <c r="B114" s="3">
-        <v>46371</v>
-      </c>
-      <c r="C114" s="1" t="s">
-        <v>304</v>
-      </c>
-      <c r="D114" s="1" t="s">
-        <v>305</v>
-      </c>
-      <c r="E114" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="F114" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="G114" s="1" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A115" s="1" t="s">
-        <v>307</v>
-      </c>
-      <c r="B115" s="3">
-        <v>46371</v>
-      </c>
-      <c r="C115" s="1" t="s">
-        <v>304</v>
-      </c>
-      <c r="D115" s="1" t="s">
-        <v>226</v>
-      </c>
-      <c r="E115" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="F115" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="G115" s="1" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A116" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="B116" s="3">
-        <v>46371</v>
-      </c>
-      <c r="C116" s="1" t="s">
-        <v>304</v>
-      </c>
-      <c r="D116" s="1" t="s">
-        <v>309</v>
-      </c>
-      <c r="E116" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="F116" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="G116" s="1" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A128" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="132" spans="1:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="A132" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B132" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C132" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="D132" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="E132" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F132" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A133" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="B133" s="3">
-        <v>46675</v>
-      </c>
-      <c r="C133" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D133" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E133" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="F133" s="1" t="s">
-        <v>311</v>
-      </c>
+      <c r="I45" s="1"/>
+      <c r="J45" s="1"/>
+      <c r="K45" s="1"/>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A48" s="2"/>
+      <c r="B48" s="2"/>
+      <c r="C48" s="2"/>
+      <c r="D48" s="2"/>
+      <c r="E48" s="2"/>
+      <c r="F48" s="2"/>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A49" s="1"/>
+      <c r="B49" s="3"/>
+      <c r="C49" s="1"/>
+      <c r="D49" s="1"/>
+      <c r="E49" s="7"/>
+      <c r="F49" s="1"/>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A50" s="1"/>
+      <c r="B50" s="3"/>
+      <c r="C50" s="1"/>
+      <c r="D50" s="1"/>
+      <c r="E50" s="7"/>
+      <c r="F50" s="1"/>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A51" s="2"/>
+      <c r="B51" s="4"/>
+      <c r="C51" s="2"/>
+      <c r="D51" s="2"/>
+      <c r="E51" s="8"/>
+      <c r="F51" s="2"/>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A59" s="2"/>
+      <c r="B59" s="2"/>
+      <c r="C59" s="2"/>
+      <c r="D59" s="2"/>
+      <c r="E59" s="2"/>
+      <c r="F59" s="2"/>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A60" s="1"/>
+      <c r="B60" s="3"/>
+      <c r="C60" s="1"/>
+      <c r="D60" s="1"/>
+      <c r="E60" s="1"/>
+      <c r="F60" s="1"/>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A61" s="1"/>
+      <c r="B61" s="3"/>
+      <c r="C61" s="1"/>
+      <c r="D61" s="1"/>
+      <c r="E61" s="1"/>
+      <c r="F61" s="1"/>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A62" s="1"/>
+      <c r="B62" s="3"/>
+      <c r="C62" s="1"/>
+      <c r="D62" s="1"/>
+      <c r="E62" s="1"/>
+      <c r="F62" s="1"/>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A63" s="1"/>
+      <c r="B63" s="3"/>
+      <c r="C63" s="1"/>
+      <c r="D63" s="1"/>
+      <c r="E63" s="1"/>
+      <c r="F63" s="1"/>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A64" s="1"/>
+      <c r="B64" s="3"/>
+      <c r="C64" s="1"/>
+      <c r="D64" s="1"/>
+      <c r="E64" s="1"/>
+      <c r="F64" s="1"/>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A65" s="1"/>
+      <c r="B65" s="3"/>
+      <c r="C65" s="1"/>
+      <c r="D65" s="1"/>
+      <c r="E65" s="1"/>
+      <c r="F65" s="1"/>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A66" s="1"/>
+      <c r="B66" s="3"/>
+      <c r="C66" s="1"/>
+      <c r="D66" s="1"/>
+      <c r="E66" s="1"/>
+      <c r="F66" s="1"/>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A67" s="1"/>
+      <c r="B67" s="3"/>
+      <c r="C67" s="1"/>
+      <c r="D67" s="1"/>
+      <c r="E67" s="1"/>
+      <c r="F67" s="1"/>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A74" s="2"/>
+      <c r="B74" s="2"/>
+      <c r="C74" s="2"/>
+      <c r="D74" s="2"/>
+      <c r="E74" s="2"/>
+      <c r="F74" s="2"/>
+      <c r="G74" s="2"/>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A75" s="1"/>
+      <c r="B75" s="3"/>
+      <c r="C75" s="1"/>
+      <c r="D75" s="1"/>
+      <c r="E75" s="1"/>
+      <c r="F75" s="1"/>
+      <c r="G75" s="1"/>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A76" s="1"/>
+      <c r="B76" s="3"/>
+      <c r="C76" s="1"/>
+      <c r="D76" s="1"/>
+      <c r="E76" s="1"/>
+      <c r="F76" s="1"/>
+      <c r="G76" s="1"/>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A77" s="1"/>
+      <c r="B77" s="3"/>
+      <c r="C77" s="1"/>
+      <c r="D77" s="1"/>
+      <c r="E77" s="1"/>
+      <c r="F77" s="1"/>
+      <c r="G77" s="1"/>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A83" s="2"/>
+      <c r="B83" s="2"/>
+      <c r="C83" s="2"/>
+      <c r="D83" s="2"/>
+      <c r="E83" s="2"/>
+      <c r="F83" s="2"/>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A84" s="1"/>
+      <c r="B84" s="3"/>
+      <c r="C84" s="1"/>
+      <c r="D84" s="1"/>
+      <c r="E84" s="1"/>
+      <c r="F84" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Prateleira: aba 28.10.26 (SOC + Acel KO + Call KO); sem PDF desta semana.
</commit_message>
<xml_diff>
--- a/prateleira/operacoes/operacoes.xlsx
+++ b/prateleira/operacoes/operacoes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PIMENTPA\Projects\Artes\clone-github\prateleira\operacoes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53304EEA-B49F-41CC-9B9C-15B30E01E882}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CA09DF8-910B-41A9-858E-71E50E630E79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15915" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{4BD3F994-188E-4AC8-9C05-940072856F1C}"/>
+    <workbookView xWindow="-15915" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{4BD3F994-188E-4AC8-9C05-940072856F1C}"/>
   </bookViews>
   <sheets>
     <sheet name="07.09.26" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="21.09.26" sheetId="3" r:id="rId3"/>
     <sheet name="28.09.26" sheetId="4" r:id="rId4"/>
     <sheet name="19.10.26" sheetId="5" r:id="rId5"/>
+    <sheet name="28.10.26" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1671" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1767" uniqueCount="336">
   <si>
     <t>SOC</t>
   </si>
@@ -976,6 +977,81 @@
   </si>
   <si>
     <t>35.63%</t>
+  </si>
+  <si>
+    <t>MBRF3</t>
+  </si>
+  <si>
+    <t>105.97%</t>
+  </si>
+  <si>
+    <t>-35.00%</t>
+  </si>
+  <si>
+    <t>AURA33</t>
+  </si>
+  <si>
+    <t>VIVT3</t>
+  </si>
+  <si>
+    <t>104.55%</t>
+  </si>
+  <si>
+    <t>-40.90%</t>
+  </si>
+  <si>
+    <t>104.05%</t>
+  </si>
+  <si>
+    <t>-43.53%</t>
+  </si>
+  <si>
+    <t>Aceleradora KO com Ativo</t>
+  </si>
+  <si>
+    <t>115.48%</t>
+  </si>
+  <si>
+    <t>-27.38%</t>
+  </si>
+  <si>
+    <t>116.33%</t>
+  </si>
+  <si>
+    <t>-26.00%</t>
+  </si>
+  <si>
+    <t>2.85%</t>
+  </si>
+  <si>
+    <t>1.45%</t>
+  </si>
+  <si>
+    <t>-30.00%</t>
+  </si>
+  <si>
+    <t>119.00%</t>
+  </si>
+  <si>
+    <t>-4.50%</t>
+  </si>
+  <si>
+    <t>16.62%</t>
+  </si>
+  <si>
+    <t>18.46%</t>
+  </si>
+  <si>
+    <t>RADL3</t>
+  </si>
+  <si>
+    <t>123.70%</t>
+  </si>
+  <si>
+    <t>118.50%</t>
+  </si>
+  <si>
+    <t>23.35%</t>
   </si>
 </sst>
 </file>
@@ -8057,4 +8133,404 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C3BA8C4-CB6C-48C5-8AEE-0FE20779D458}">
+  <dimension ref="A1:H17"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.26953125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" s="1"/>
+      <c r="B2" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="C2" s="4">
+        <v>46353</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" s="1"/>
+      <c r="B3" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="C3" s="4">
+        <v>46353</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" s="1"/>
+      <c r="B4" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="C4" s="4">
+        <v>46370</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" s="1"/>
+      <c r="B5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="4">
+        <v>46370</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+    </row>
+    <row r="7" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" s="1"/>
+      <c r="B8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" s="4">
+        <v>46443</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" s="1"/>
+      <c r="B9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="4">
+        <v>46443</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" s="1"/>
+      <c r="B10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="4">
+        <v>46413</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" s="1"/>
+      <c r="B11" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C11" s="4">
+        <v>46413</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+    </row>
+    <row r="13" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A14" s="1"/>
+      <c r="B14" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C14" s="4">
+        <v>46384</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A15" s="1"/>
+      <c r="B15" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="C15" s="4">
+        <v>46384</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A16" s="1"/>
+      <c r="B16" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="C16" s="4">
+        <v>46384</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A17" s="1"/>
+      <c r="B17" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C17" s="4">
+        <v>46384</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>335</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Prateleira: aba 28.10 - Aceleradora ITUB4 KO 114.75, remove AXIA3.
</commit_message>
<xml_diff>
--- a/prateleira/operacoes/operacoes.xlsx
+++ b/prateleira/operacoes/operacoes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PIMENTPA\Projects\Artes\clone-github\prateleira\operacoes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CA09DF8-910B-41A9-858E-71E50E630E79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{099460C3-6862-43C1-AA22-F470693AF4D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-15915" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{4BD3F994-188E-4AC8-9C05-940072856F1C}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1767" uniqueCount="336">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1761" uniqueCount="334">
   <si>
     <t>SOC</t>
   </si>
@@ -1009,18 +1009,9 @@
     <t>Aceleradora KO com Ativo</t>
   </si>
   <si>
-    <t>115.48%</t>
-  </si>
-  <si>
     <t>-27.38%</t>
   </si>
   <si>
-    <t>116.33%</t>
-  </si>
-  <si>
-    <t>-26.00%</t>
-  </si>
-  <si>
     <t>2.85%</t>
   </si>
   <si>
@@ -1052,6 +1043,9 @@
   </si>
   <si>
     <t>23.35%</t>
+  </si>
+  <si>
+    <t>114.75%</t>
   </si>
 </sst>
 </file>
@@ -8137,7 +8131,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C3BA8C4-CB6C-48C5-8AEE-0FE20779D458}">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.453125" bestFit="1" customWidth="1"/>
@@ -8311,49 +8305,49 @@
         <v>46443</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>292</v>
+        <v>64</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="1"/>
       <c r="B9" s="2" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="C9" s="4">
-        <v>46443</v>
+        <v>46413</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>292</v>
+        <v>64</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>323</v>
+        <v>185</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>323</v>
+        <v>185</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>15</v>
+        <v>322</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>324</v>
+        <v>186</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="1"/>
       <c r="B10" s="2" t="s">
-        <v>25</v>
+        <v>80</v>
       </c>
       <c r="C10" s="4">
         <v>46413</v>
@@ -8368,76 +8362,76 @@
         <v>185</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>186</v>
+        <v>324</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="1"/>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+    </row>
+    <row r="12" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" s="1"/>
+      <c r="B13" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C11" s="4">
-        <v>46413</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="G11" s="2" t="s">
+      <c r="C13" s="4">
+        <v>46384</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>326</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H13" s="2" t="s">
         <v>327</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
-    </row>
-    <row r="13" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="1"/>
       <c r="B14" s="2" t="s">
-        <v>80</v>
+        <v>265</v>
       </c>
       <c r="C14" s="4">
         <v>46384</v>
@@ -8446,22 +8440,22 @@
         <v>64</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>328</v>
+        <v>95</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>52</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="1"/>
       <c r="B15" s="2" t="s">
-        <v>265</v>
+        <v>329</v>
       </c>
       <c r="C15" s="4">
         <v>46384</v>
@@ -8470,22 +8464,22 @@
         <v>64</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>95</v>
+        <v>330</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>52</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>331</v>
+        <v>294</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
       <c r="B16" s="2" t="s">
-        <v>332</v>
+        <v>175</v>
       </c>
       <c r="C16" s="4">
         <v>46384</v>
@@ -8494,40 +8488,16 @@
         <v>64</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>52</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A17" s="1"/>
-      <c r="B17" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="C17" s="4">
-        <v>46384</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>334</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>329</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
     </row>
   </sheetData>

</xml_diff>